<commit_message>
feat (data_siswa_example.xlsx) : udd kartu_keluarga Column
</commit_message>
<xml_diff>
--- a/data_siswa_example.xlsx
+++ b/data_siswa_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\laragon\www\python\emis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E66F11-0B82-4BDA-97F7-ED129AFE201A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E14ABBA-BD5F-43E2-9E80-DA96333FBC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E3F6456E-2CF0-407C-BCF5-C11B6929A961}"/>
   </bookViews>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>full_name</t>
   </si>
@@ -246,7 +246,7 @@
     <t>status</t>
   </si>
   <si>
-    <t>m_residence_status_id2</t>
+    <t>kartu_keluarga</t>
   </si>
 </sst>
 </file>
@@ -256,7 +256,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="8"/>
       <color theme="1"/>
@@ -283,16 +283,43 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -300,24 +327,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="3">
     <dxf>
       <border>
         <left style="thin">
@@ -352,15 +432,6 @@
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -413,52 +484,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F2519E9-2327-44F7-991B-A73393265A96}" name="Table1" displayName="Table1" ref="A1:AK2" totalsRowShown="0">
-  <autoFilter ref="A1:AK2" xr:uid="{1F2519E9-2327-44F7-991B-A73393265A96}"/>
-  <tableColumns count="37">
-    <tableColumn id="1" xr3:uid="{EB8F8004-EA0F-43A8-9393-34C34A750558}" name="full_name"/>
-    <tableColumn id="2" xr3:uid="{3B157DE6-B351-4285-8EC2-E780FD881C04}" name="nik"/>
-    <tableColumn id="3" xr3:uid="{6CCD1380-57E4-4A10-A401-1188C419B85F}" name="gender"/>
-    <tableColumn id="4" xr3:uid="{752E82C8-A7D0-4310-827B-D3FBF74A6534}" name="birth_place"/>
-    <tableColumn id="5" xr3:uid="{7C9E90DD-52D1-429C-883E-57BC84FA04B4}" name="birth_date" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{9B60332A-1BEC-42C0-9BF3-D15793BB2C24}" name="siblings_num"/>
-    <tableColumn id="7" xr3:uid="{252FA5E9-6651-4F81-A530-FE2A1D7DCE72}" name="child_of_num"/>
-    <tableColumn id="8" xr3:uid="{8E266A14-795F-4927-BC4E-BF65935706E1}" name="m_residence_status_id"/>
-    <tableColumn id="9" xr3:uid="{24E13680-3099-4DCA-9590-6D3516466956}" name="m_province_id"/>
-    <tableColumn id="10" xr3:uid="{6339AA14-E2C0-4395-AB7A-106837BC2FCC}" name="m_city_id"/>
-    <tableColumn id="11" xr3:uid="{D6DCBF4D-0289-402A-9F13-14E09D343C6A}" name="m_district_id"/>
-    <tableColumn id="12" xr3:uid="{F57ABD42-95FA-4F21-BB93-953B9CB86725}" name="m_subdistrict_id"/>
-    <tableColumn id="13" xr3:uid="{B5474311-7E94-4047-8FE6-63B4A8B32508}" name="address"/>
-    <tableColumn id="14" xr3:uid="{813F4F43-BE1B-4ED3-A43A-5F63E3F6FDDF}" name="postal_code_num"/>
-    <tableColumn id="15" xr3:uid="{12D1B521-83D3-4A7F-8E2F-9DC6A73D5C57}" name="m_level_id"/>
-    <tableColumn id="16" xr3:uid="{B8E57E6B-156E-435E-8470-AFC3D18BC067}" name="kk_num"/>
-    <tableColumn id="17" xr3:uid="{789E5CF5-2D86-420C-A692-7AF91265806F}" name="family_head_name"/>
-    <tableColumn id="18" xr3:uid="{10E222D9-FC48-491A-AB7B-91DAFD391F5A}" name="father_full_name"/>
-    <tableColumn id="19" xr3:uid="{C2BCC7F1-CD70-4103-8237-0EEA4AF6ECC4}" name="father_m_life_status_id"/>
-    <tableColumn id="20" xr3:uid="{491D20CE-0AD1-4A72-BDF6-4F25A74D473B}" name="father_nik"/>
-    <tableColumn id="21" xr3:uid="{A4B5512B-4912-4B6F-A513-A82B0FC98F9B}" name="father_birth_place"/>
-    <tableColumn id="22" xr3:uid="{F6EDCAA2-A3C5-4A85-BC3C-FA34FE7E1854}" name="father_birth_date" dataDxfId="4"/>
-    <tableColumn id="23" xr3:uid="{18C41F0A-550D-4BBD-B30C-F87C2FDD495A}" name="father_m_last_education_id"/>
-    <tableColumn id="24" xr3:uid="{7360FB9F-530D-42A7-A835-F313A3E7D7BB}" name="father_m_job_id"/>
-    <tableColumn id="25" xr3:uid="{229F121C-AC67-4E93-857A-1CA4E6BD7485}" name="father_m_average_income_per_month_id"/>
-    <tableColumn id="26" xr3:uid="{612EDA71-35CB-48EF-95C1-287F8A80E520}" name="father_phone_number"/>
-    <tableColumn id="27" xr3:uid="{4AE4322D-2E06-444D-B31F-214F60EF6FB1}" name="mother_m_life_status_id"/>
-    <tableColumn id="28" xr3:uid="{CB3E7E98-77A9-4ADA-80D3-7408346CDAA9}" name="mother_full_name"/>
-    <tableColumn id="29" xr3:uid="{4EF710B9-ED00-45F0-A4BC-DF5F2F076D91}" name="mother_nik"/>
-    <tableColumn id="30" xr3:uid="{D7A92AAF-F769-47AE-84B0-04A468BB44CE}" name="mother_birth_place"/>
-    <tableColumn id="31" xr3:uid="{7E69F2D3-A81D-4E5C-9085-3CA005FDC85B}" name="mother_birth_date" dataDxfId="3"/>
-    <tableColumn id="32" xr3:uid="{6D64A2BF-097B-4588-8BF5-D4B826F950B5}" name="mother_m_last_education_id"/>
-    <tableColumn id="33" xr3:uid="{E4F0FC64-3031-4C78-93D3-248A63EF2E7B}" name="mother_m_job_id"/>
-    <tableColumn id="34" xr3:uid="{57C032A4-83CD-4316-8165-38D478220A38}" name="mother_m_average_income_per_month_id"/>
-    <tableColumn id="35" xr3:uid="{C6770FA1-1834-486B-B204-0D013F2EA1DE}" name="mother_phone_number"/>
-    <tableColumn id="36" xr3:uid="{4B3DA0AE-638C-469B-B57C-B92A77F71DA9}" name="m_residence_status_id2"/>
-    <tableColumn id="37" xr3:uid="{EDE2A089-F090-480F-B038-AB6B4997DEE5}" name="status"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -778,14 +803,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E139DADF-622C-4753-A394-6ADA81141C75}">
-  <dimension ref="A1:AK1"/>
+  <dimension ref="A1:AL2"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
     <col min="2" max="2" width="20.5" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" style="4" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
@@ -801,7 +826,7 @@
     <col min="18" max="18" width="41.6640625" customWidth="1"/>
     <col min="19" max="19" width="25" customWidth="1"/>
     <col min="20" max="21" width="31.5" customWidth="1"/>
-    <col min="22" max="22" width="31.5" style="5" customWidth="1"/>
+    <col min="22" max="22" width="31.5" style="4" customWidth="1"/>
     <col min="23" max="23" width="31.5" customWidth="1"/>
     <col min="24" max="24" width="23.33203125" customWidth="1"/>
     <col min="25" max="25" width="41.6640625" customWidth="1"/>
@@ -810,7 +835,7 @@
     <col min="28" max="28" width="20.1640625" customWidth="1"/>
     <col min="29" max="29" width="21.83203125" customWidth="1"/>
     <col min="30" max="30" width="26.33203125" customWidth="1"/>
-    <col min="31" max="31" width="20.5" style="5" customWidth="1"/>
+    <col min="31" max="31" width="20.5" style="4" customWidth="1"/>
     <col min="32" max="32" width="30" customWidth="1"/>
     <col min="33" max="33" width="23.33203125" customWidth="1"/>
     <col min="34" max="34" width="43" customWidth="1"/>
@@ -865,118 +890,161 @@
     <col min="84" max="84" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AE1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="AK1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="AK1" t="s">
-        <v>35</v>
-      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
+      <c r="AE2" s="14"/>
+      <c r="AF2" s="13"/>
+      <c r="AG2" s="13"/>
+      <c r="AH2" s="13"/>
+      <c r="AI2" s="13"/>
+      <c r="AJ2" s="13"/>
+      <c r="AK2" s="13"/>
+      <c r="AL2" s="13"/>
     </row>
   </sheetData>
   <dataValidations count="23">
@@ -1010,9 +1078,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1025,27 +1090,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4">
+      <c r="A1" s="3">
         <v>35384</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>34931</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>33774</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>34285</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
+      <c r="A5" s="2"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>

</xml_diff>